<commit_message>
Q2 2026 Fiscal Update
</commit_message>
<xml_diff>
--- a/Data/Fiscal Data/BIR-Tax-Statistics.xlsx
+++ b/Data/Fiscal Data/BIR-Tax-Statistics.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AJ\GitHub Repositories\PH-Econ-Data\Data\Fiscal Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7311032A-23BC-4CB5-8A9B-FA5158B8D9F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F374FCD1-9318-4C02-8629-E5AA9F1607DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="765" yWindow="1470" windowWidth="15270" windowHeight="11610" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12105" yWindow="1845" windowWidth="15780" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="By Source, Millions" sheetId="1" r:id="rId1"/>
@@ -1131,11 +1131,11 @@
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="4" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="4" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="4" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="4" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="4" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="4" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1652,9 +1652,11 @@
       <c r="A2" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="B2" s="2"/>
+      <c r="B2" s="2">
+        <v>3109828.54</v>
+      </c>
       <c r="C2" s="2">
-        <v>3232475.0260000001</v>
+        <v>3101900</v>
       </c>
       <c r="D2" s="2">
         <v>2851603.73</v>
@@ -1916,15 +1918,19 @@
       <c r="A3" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2">
-        <v>1711755.2549999999</v>
-      </c>
-      <c r="D3" s="2">
+      <c r="B3" s="12">
+        <f t="shared" ref="B3:C3" si="0">SUM(B4,B7,B12)</f>
+        <v>1687012.2199999997</v>
+      </c>
+      <c r="C3" s="12">
+        <f t="shared" si="0"/>
+        <v>1683967.1400000001</v>
+      </c>
+      <c r="D3" s="12">
         <f>SUM(D4,D7,D12)</f>
         <v>1532764.6</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="12">
         <f>SUM(E4,E7,E12)</f>
         <v>1553411.6600000001</v>
       </c>
@@ -2166,8 +2172,12 @@
       <c r="A4" t="s">
         <v>84</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
+      <c r="B4" s="3">
+        <v>685375.48</v>
+      </c>
+      <c r="C4" s="3">
+        <v>636555.18999999994</v>
+      </c>
       <c r="D4" s="3">
         <v>583710.06000000006</v>
       </c>
@@ -2404,8 +2414,12 @@
       <c r="A5" t="s">
         <v>85</v>
       </c>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
+      <c r="B5" s="3">
+        <v>377768.93</v>
+      </c>
+      <c r="C5" s="3">
+        <v>373254.77</v>
+      </c>
       <c r="D5" s="3">
         <v>335216.42</v>
       </c>
@@ -2642,8 +2656,12 @@
       <c r="A6" t="s">
         <v>86</v>
       </c>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
+      <c r="B6" s="3">
+        <v>307606.55</v>
+      </c>
+      <c r="C6" s="3">
+        <v>263300.43</v>
+      </c>
       <c r="D6" s="3">
         <v>248493.63</v>
       </c>
@@ -2880,8 +2898,12 @@
       <c r="A7" t="s">
         <v>87</v>
       </c>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
+      <c r="B7" s="3">
+        <v>809066.61</v>
+      </c>
+      <c r="C7" s="3">
+        <v>849482.93</v>
+      </c>
       <c r="D7" s="3">
         <v>764632.9</v>
       </c>
@@ -3114,8 +3136,12 @@
       <c r="A8" t="s">
         <v>88</v>
       </c>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
+      <c r="B8" s="3">
+        <v>29327.74</v>
+      </c>
+      <c r="C8" s="3">
+        <v>26092.98</v>
+      </c>
       <c r="D8" s="3">
         <v>23287.56</v>
       </c>
@@ -3348,8 +3374,12 @@
       <c r="A9" t="s">
         <v>89</v>
       </c>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
+      <c r="B9" s="3">
+        <v>411349.69</v>
+      </c>
+      <c r="C9" s="3">
+        <v>401356.81</v>
+      </c>
       <c r="D9" s="3">
         <v>364454.33</v>
       </c>
@@ -3582,8 +3612,12 @@
       <c r="A10" t="s">
         <v>90</v>
       </c>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
+      <c r="B10" s="3">
+        <v>34871.5</v>
+      </c>
+      <c r="C10" s="3">
+        <v>36775.81</v>
+      </c>
       <c r="D10" s="3">
         <v>34478.22</v>
       </c>
@@ -3800,8 +3834,12 @@
       <c r="A11" t="s">
         <v>91</v>
       </c>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
+      <c r="B11" s="3">
+        <v>333517.68</v>
+      </c>
+      <c r="C11" s="3">
+        <v>385257.33</v>
+      </c>
       <c r="D11" s="3">
         <v>342412.78</v>
       </c>
@@ -4014,8 +4052,14 @@
       <c r="A12" t="s">
         <v>92</v>
       </c>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
+      <c r="B12" s="11">
+        <f t="shared" ref="B12:C12" si="1">SUM(B13:B14)</f>
+        <v>192570.13</v>
+      </c>
+      <c r="C12" s="11">
+        <f t="shared" si="1"/>
+        <v>197929.02</v>
+      </c>
       <c r="D12" s="11">
         <f>SUM(D13:D14)</f>
         <v>184421.64</v>
@@ -4238,8 +4282,12 @@
       <c r="A13" t="s">
         <v>93</v>
       </c>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
+      <c r="B13" s="3">
+        <v>99351.1</v>
+      </c>
+      <c r="C13" s="3">
+        <v>104418.79</v>
+      </c>
       <c r="D13" s="3">
         <v>107354.21</v>
       </c>
@@ -4456,8 +4504,12 @@
       <c r="A14" t="s">
         <v>94</v>
       </c>
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
+      <c r="B14" s="11">
+        <v>93219.03</v>
+      </c>
+      <c r="C14" s="11">
+        <v>93510.23</v>
+      </c>
       <c r="D14" s="11">
         <v>77067.429999999993</v>
       </c>
@@ -5072,9 +5124,11 @@
       <c r="A19" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="B19" s="2"/>
+      <c r="B19" s="2">
+        <v>327156.34000000003</v>
+      </c>
       <c r="C19" s="2">
-        <v>343103.80699999997</v>
+        <v>328898.06</v>
       </c>
       <c r="D19" s="2">
         <v>304279.07</v>
@@ -5320,9 +5374,11 @@
       <c r="A20" t="s">
         <v>100</v>
       </c>
-      <c r="B20" s="3"/>
+      <c r="B20" s="3">
+        <v>121213.49</v>
+      </c>
       <c r="C20" s="3">
-        <v>130038</v>
+        <v>122235.13</v>
       </c>
       <c r="D20" s="3">
         <v>116088.08</v>
@@ -5544,9 +5600,11 @@
       <c r="A21" t="s">
         <v>101</v>
       </c>
-      <c r="B21" s="3"/>
+      <c r="B21" s="3">
+        <v>150902.68</v>
+      </c>
       <c r="C21" s="3">
-        <v>148920</v>
+        <v>149570.70000000001</v>
       </c>
       <c r="D21" s="3">
         <v>134433.13</v>
@@ -5768,7 +5826,9 @@
       <c r="A22" t="s">
         <v>102</v>
       </c>
-      <c r="B22" s="3"/>
+      <c r="B22" s="3">
+        <v>134.21</v>
+      </c>
       <c r="C22" s="3"/>
       <c r="D22" s="3">
         <v>98.15</v>
@@ -5984,8 +6044,12 @@
       <c r="A23" t="s">
         <v>103</v>
       </c>
-      <c r="B23" s="3"/>
-      <c r="C23" s="3"/>
+      <c r="B23" s="3">
+        <v>42462.94</v>
+      </c>
+      <c r="C23" s="3">
+        <v>46202.01</v>
+      </c>
       <c r="D23" s="3">
         <v>43690.83</v>
       </c>
@@ -6206,9 +6270,11 @@
       <c r="A24" t="s">
         <v>330</v>
       </c>
-      <c r="B24" s="3"/>
+      <c r="B24" s="3">
+        <v>36402.269999999997</v>
+      </c>
       <c r="C24" s="3">
-        <v>39279</v>
+        <v>39708.89</v>
       </c>
       <c r="D24" s="3">
         <v>37638.75</v>
@@ -6231,25 +6297,25 @@
       <c r="J24" s="3">
         <v>32950.94</v>
       </c>
-      <c r="K24" s="14">
+      <c r="K24" s="13">
         <v>34043</v>
       </c>
-      <c r="L24" s="15">
+      <c r="L24" s="14">
         <v>32417.759999999998</v>
       </c>
-      <c r="M24" s="14">
+      <c r="M24" s="13">
         <v>28617</v>
       </c>
-      <c r="N24" s="15">
+      <c r="N24" s="14">
         <v>38622.83</v>
       </c>
-      <c r="O24" s="14">
+      <c r="O24" s="13">
         <v>37286</v>
       </c>
-      <c r="P24" s="15">
+      <c r="P24" s="14">
         <v>35510.589999999997</v>
       </c>
-      <c r="Q24" s="14">
+      <c r="Q24" s="13">
         <v>46455</v>
       </c>
       <c r="R24" s="3"/>
@@ -6328,9 +6394,11 @@
       <c r="A25" t="s">
         <v>104</v>
       </c>
-      <c r="B25" s="3"/>
+      <c r="B25" s="3">
+        <v>12443.02</v>
+      </c>
       <c r="C25" s="3">
-        <v>11070</v>
+        <v>10890.22</v>
       </c>
       <c r="D25" s="3">
         <v>9968.8700000000008</v>
@@ -6916,9 +6984,11 @@
       <c r="A29" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="B29" s="2"/>
+      <c r="B29" s="2">
+        <v>679797.75</v>
+      </c>
       <c r="C29" s="2">
-        <v>710042.87100000004</v>
+        <v>707430.62</v>
       </c>
       <c r="D29" s="2">
         <v>643846.18999999994</v>
@@ -7142,9 +7212,11 @@
       <c r="A30" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="B30" s="2"/>
+      <c r="B30" s="2">
+        <v>144982.85</v>
+      </c>
       <c r="C30" s="2">
-        <v>178464.02600000001</v>
+        <v>125050.61</v>
       </c>
       <c r="D30" s="2">
         <v>136324.25</v>
@@ -7390,8 +7462,12 @@
       <c r="A31" t="s">
         <v>110</v>
       </c>
-      <c r="B31" s="3"/>
-      <c r="C31" s="3"/>
+      <c r="B31" s="3">
+        <v>92840.91</v>
+      </c>
+      <c r="C31" s="3">
+        <v>87686.25</v>
+      </c>
       <c r="D31" s="3">
         <v>71687.17</v>
       </c>
@@ -7612,8 +7688,12 @@
       <c r="A32" t="s">
         <v>111</v>
       </c>
-      <c r="B32" s="3"/>
-      <c r="C32" s="3"/>
+      <c r="B32" s="3">
+        <v>4105.04</v>
+      </c>
+      <c r="C32" s="3">
+        <v>5291.06</v>
+      </c>
       <c r="D32" s="3">
         <v>14179.1</v>
       </c>
@@ -7834,8 +7914,12 @@
       <c r="A33" t="s">
         <v>112</v>
       </c>
-      <c r="B33" s="3"/>
-      <c r="C33" s="3"/>
+      <c r="B33" s="3">
+        <v>810.02</v>
+      </c>
+      <c r="C33" s="3">
+        <v>497</v>
+      </c>
       <c r="D33" s="3">
         <v>414.66</v>
       </c>
@@ -8056,8 +8140,12 @@
       <c r="A34" t="s">
         <v>113</v>
       </c>
-      <c r="B34" s="3"/>
-      <c r="C34" s="3"/>
+      <c r="B34" s="3">
+        <v>45714.720000000001</v>
+      </c>
+      <c r="C34" s="3">
+        <v>31337.13</v>
+      </c>
       <c r="D34" s="3">
         <v>49866.57</v>
       </c>
@@ -8278,8 +8366,12 @@
       <c r="A35" t="s">
         <v>114</v>
       </c>
-      <c r="B35" s="3"/>
-      <c r="C35" s="3"/>
+      <c r="B35" s="3">
+        <v>1512.16</v>
+      </c>
+      <c r="C35" s="3">
+        <v>239.16</v>
+      </c>
       <c r="D35" s="3">
         <v>176.74</v>
       </c>
@@ -8650,9 +8742,13 @@
       <c r="A37" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="B37" s="2"/>
-      <c r="C37" s="2">
-        <v>289109.06699999998</v>
+      <c r="B37" s="12">
+        <f t="shared" ref="B37:C37" si="2">SUM(B38:B41)</f>
+        <v>270879.37</v>
+      </c>
+      <c r="C37" s="12">
+        <f t="shared" si="2"/>
+        <v>256553.58</v>
       </c>
       <c r="D37" s="12">
         <f>SUM(D38:D41)</f>
@@ -8901,8 +8997,12 @@
       <c r="A38" t="s">
         <v>117</v>
       </c>
-      <c r="B38" s="3"/>
-      <c r="C38" s="3"/>
+      <c r="B38" s="3">
+        <v>18504.310000000001</v>
+      </c>
+      <c r="C38" s="3">
+        <v>12045</v>
+      </c>
       <c r="D38" s="3">
         <v>11096.92</v>
       </c>
@@ -9143,8 +9243,14 @@
       <c r="A39" t="s">
         <v>118</v>
       </c>
-      <c r="B39" s="3"/>
-      <c r="C39" s="3"/>
+      <c r="B39" s="11">
+        <f>189447.99+25037.47</f>
+        <v>214485.46</v>
+      </c>
+      <c r="C39" s="11">
+        <f>193818.21+20947</f>
+        <v>214765.21</v>
+      </c>
       <c r="D39" s="11">
         <f>177337.99+19536.16</f>
         <v>196874.15</v>
@@ -9579,8 +9685,12 @@
       <c r="A41" t="s">
         <v>120</v>
       </c>
-      <c r="B41" s="3"/>
-      <c r="C41" s="3"/>
+      <c r="B41" s="3">
+        <v>37889.599999999999</v>
+      </c>
+      <c r="C41" s="3">
+        <v>29743.37</v>
+      </c>
       <c r="D41" s="3">
         <v>26418.560000000001</v>
       </c>
@@ -11867,7 +11977,7 @@
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="15" t="s">
         <v>134</v>
       </c>
       <c r="B4" s="4" t="s">
@@ -11875,19 +11985,19 @@
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="13"/>
+      <c r="A5" s="15"/>
       <c r="B5" s="4" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="13"/>
+      <c r="A6" s="15"/>
       <c r="B6" s="4" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="13"/>
+      <c r="A7" s="15"/>
       <c r="B7" s="4"/>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>